<commit_message>
Modification CAD Ajout fixation capot
</commit_message>
<xml_diff>
--- a/BOM_LignePassionIIm.xlsx
+++ b/BOM_LignePassionIIm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79fc430203973324/TravauxMetriques/IIm/Passion IIm/PupitreLigne/AlimLigne_PassionIIm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a43dc3239fed0de/PCB_Perso/PCB_IIm_Ligne/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="445" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0044CF36-3191-4FF6-82AC-6BD1CA97D11B}"/>
+  <xr:revisionPtr revIDLastSave="456" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B761E83-DB32-4B38-B85C-1E82C14F5181}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -657,6 +657,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -684,8 +686,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
@@ -1180,36 +1180,36 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B7EC6F-57FE-4577-A1D4-89717E48955F}">
   <dimension ref="A1:M44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" customWidth="1"/>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="12.77734375" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="9" max="9" width="12.109375" customWidth="1"/>
-    <col min="10" max="10" width="19.88671875" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" customWidth="1"/>
-    <col min="12" max="12" width="79.5546875" customWidth="1"/>
+    <col min="1" max="1" width="25.53125" customWidth="1"/>
+    <col min="2" max="2" width="18.1328125" customWidth="1"/>
+    <col min="3" max="3" width="12.796875" customWidth="1"/>
+    <col min="4" max="4" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.86328125" customWidth="1"/>
+    <col min="9" max="9" width="12.1328125" customWidth="1"/>
+    <col min="10" max="10" width="19.86328125" customWidth="1"/>
+    <col min="11" max="11" width="12.46484375" customWidth="1"/>
+    <col min="12" max="12" width="79.53125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A1" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-    </row>
-    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="18"/>
+      <c r="J1" s="18"/>
+      <c r="K1" s="18"/>
+      <c r="L1" s="18"/>
+    </row>
+    <row r="2" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
@@ -1250,7 +1250,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1273,7 +1273,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -1295,7 +1295,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>106</v>
       </c>
@@ -1319,11 +1319,11 @@
       <c r="K5" t="s">
         <v>54</v>
       </c>
-      <c r="L5" t="s">
+      <c r="L5" s="14" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -1347,11 +1347,11 @@
       <c r="K6" t="s">
         <v>54</v>
       </c>
-      <c r="L6" t="s">
+      <c r="L6" s="14" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1369,11 +1369,11 @@
       <c r="K7" t="s">
         <v>54</v>
       </c>
-      <c r="L7" t="s">
+      <c r="L7" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1395,7 +1395,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -1413,11 +1413,11 @@
       <c r="K9" t="s">
         <v>54</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="14" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -1439,7 +1439,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1460,11 +1460,11 @@
       <c r="K11" t="s">
         <v>54</v>
       </c>
-      <c r="L11" t="s">
+      <c r="L11" s="14" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>72</v>
       </c>
@@ -1482,11 +1482,11 @@
       <c r="K12" t="s">
         <v>54</v>
       </c>
-      <c r="L12" t="s">
+      <c r="L12" s="14" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1508,7 +1508,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -1551,11 +1551,11 @@
       <c r="K15" t="s">
         <v>54</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L15" s="14" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -1618,7 +1618,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>58</v>
       </c>
@@ -1640,7 +1640,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>555</v>
       </c>
@@ -1678,7 +1678,7 @@
       <c r="E20" t="s">
         <v>34</v>
       </c>
-      <c r="F20" s="25">
+      <c r="F20" s="16">
         <v>1</v>
       </c>
       <c r="H20" s="2">
@@ -1701,7 +1701,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1714,7 +1714,7 @@
       <c r="E21" t="s">
         <v>38</v>
       </c>
-      <c r="F21" s="25">
+      <c r="F21" s="16">
         <v>3</v>
       </c>
       <c r="H21" s="2">
@@ -1737,7 +1737,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1750,7 +1750,7 @@
       <c r="E22" t="s">
         <v>41</v>
       </c>
-      <c r="F22" s="25">
+      <c r="F22" s="16">
         <v>1</v>
       </c>
       <c r="H22" s="2">
@@ -1773,7 +1773,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -1786,7 +1786,7 @@
       <c r="E23" t="s">
         <v>99</v>
       </c>
-      <c r="F23" s="25">
+      <c r="F23" s="16">
         <v>1</v>
       </c>
       <c r="H23" s="2">
@@ -1809,7 +1809,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -1823,7 +1823,7 @@
       <c r="E24" t="s">
         <v>18</v>
       </c>
-      <c r="F24" s="25">
+      <c r="F24" s="16">
         <v>4</v>
       </c>
       <c r="H24" s="2">
@@ -1846,7 +1846,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>113</v>
       </c>
@@ -1859,7 +1859,7 @@
       <c r="E25" t="s">
         <v>115</v>
       </c>
-      <c r="F25" s="25">
+      <c r="F25" s="16">
         <v>1</v>
       </c>
       <c r="H25" s="2">
@@ -1880,7 +1880,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>84</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -1948,7 +1948,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1973,7 +1973,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -1998,7 +1998,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -2023,7 +2023,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -2048,7 +2048,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -2073,7 +2073,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2097,7 +2097,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>20</v>
       </c>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2137,11 +2137,11 @@
       </c>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
         <v>29</v>
       </c>
@@ -2149,16 +2149,16 @@
       <c r="C38" s="8">
         <v>46126</v>
       </c>
-      <c r="D38" s="17" t="e" vm="1">
+      <c r="D38" s="19" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="E38" s="18"/>
-      <c r="F38" s="19"/>
+      <c r="E38" s="20"/>
+      <c r="F38" s="21"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
-      <c r="J38" s="26"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="J38" s="17"/>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="7" t="s">
         <v>28</v>
       </c>
@@ -2166,13 +2166,13 @@
       <c r="C39" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D39" s="20"/>
-      <c r="E39" s="16"/>
-      <c r="F39" s="21"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="23"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="7" t="s">
         <v>30</v>
       </c>
@@ -2180,11 +2180,11 @@
       <c r="C40" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D40" s="20"/>
-      <c r="E40" s="16"/>
-      <c r="F40" s="21"/>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D40" s="22"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="23"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41" s="10" t="s">
         <v>31</v>
       </c>
@@ -2192,19 +2192,19 @@
       <c r="C41" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D41" s="22"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="24"/>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="D41" s="24"/>
+      <c r="E41" s="25"/>
+      <c r="F41" s="26"/>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
     </row>
@@ -2217,11 +2217,18 @@
     <hyperlink ref="L16" r:id="rId1" xr:uid="{B3065FAB-E838-4A51-A82F-630335C42D81}"/>
     <hyperlink ref="L24" r:id="rId2" xr:uid="{2207D865-CE83-4458-802D-86175171E33D}"/>
     <hyperlink ref="L18" r:id="rId3" display="https://www.conrad.ch/de/p/tru-components-tc-13895648-rundsteckverbinder-stecker-buchsenkontakt-gesamtpolzahl-6-serie-rundsteckverbinder-gx16-3473912.html?insert=UP&amp;WT.srch=1&amp;ef_id=CjwKCAjw5s_QBhAdEiwADD_gBlB0NtPFlP1PxWWOBrmvbSo2JJn5T44wcE8r8-Hav4RDqu4GGAYJ1RoCRWEQAvD_BwE:G:s" xr:uid="{D4E7E61F-AE6E-48A3-9576-9A9FC4F56721}"/>
+    <hyperlink ref="L5" r:id="rId4" display="https://de.aliexpress.com/item/1005005674103930.html?spm=a2g0o.productlist.main.1.637ejuNajuNa2p&amp;algo_pvid=b22cab55-934f-49f0-ab1c-9d69b66ca252&amp;pdp_ext_f=%7B%22order%22%3A%223052%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005005674103930%7C_p_origin_prod%3A" xr:uid="{2788E9F2-0F46-41F5-A719-257754312229}"/>
+    <hyperlink ref="L6" r:id="rId5" display="https://de.aliexpress.com/item/1005004002774546.html?spm=a2g0o.productlist.main.6.18ab20bbmHcGED&amp;aem_p4p_detail=202608121236371154182288705600000113625&amp;algo_pvid=00e039e6-f960-4780-bcc3-bce9310ef85b&amp;pdp_ext_f=%7B%22order%22%3A%222407%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005004002774546%7C_p_origin_prod%3A&amp;search_p4p_id=202608121236371154182288705600000113625_10" xr:uid="{1AD0CD3E-B953-491E-BFBE-D10DCE21EAAE}"/>
+    <hyperlink ref="L7" r:id="rId6" display="https://de.aliexpress.com/item/1005011562556892.html?spm=a2g0o.productlist.main.16.6cc12ea0bxeVQp&amp;utparam-url=scene%3Asearch%7Cquery_from%3Apc_back_same_best%7Cx_object_id%3A1005011562556892%7C_p_origin_prod%3A&amp;algo_pvid=50ab7cf4-e162-4535-b9d9-a2be6ca5b335&amp;pdp_ext_f=%7B%22order%22%3A%227%22%2C%22fromPage%22%3A%22search%22%7D" xr:uid="{119994E1-3262-4B32-920D-09A1CD88AE8E}"/>
+    <hyperlink ref="L9" r:id="rId7" display="https://de.aliexpress.com/item/1005011562556892.html?spm=a2g0o.productlist.main.16.6cc12ea0bxeVQp&amp;utparam-url=scene%3Asearch%7Cquery_from%3Apc_back_same_best%7Cx_object_id%3A1005011562556892%7C_p_origin_prod%3A&amp;algo_pvid=50ab7cf4-e162-4535-b9d9-a2be6ca5b335&amp;pdp_ext_f=%7B%22order%22%3A%227%22%2C%22fromPage%22%3A%22search%22%7D" xr:uid="{14976960-CF54-41FA-BD6E-64D5F5097F11}"/>
+    <hyperlink ref="L11" r:id="rId8" display="https://de.aliexpress.com/item/1005012410174447.html?spm=a2g0o.productlist.main.3.1c57pPLrpPLrXF&amp;algo_pvid=8d846d87-e1c7-4911-9404-42bf57029f2f&amp;pdp_ext_f=%7B%22order%22%3A%223%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005012410174447%7C_p_origin_prod%3A" xr:uid="{4167C8F0-16BB-4349-AB96-8D1E7EA17B0B}"/>
+    <hyperlink ref="L12" r:id="rId9" display="https://de.aliexpress.com/item/1005008777027854.html?spm=a2g0o.productlist.main.3.34a9f054Jnh2d5&amp;algo_pvid=a3217470-cd61-4707-8b2f-7d76497918d0&amp;pdp_ext_f=%7B%22order%22%3A%221295%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005008777027854%7C_p_origin_prod%3A" xr:uid="{E1DCA1E5-10CE-4744-82AE-57A8AEE1E4BC}"/>
+    <hyperlink ref="L15" r:id="rId10" display="https://de.aliexpress.com/item/32676786935.html?spm=a2g0o.productlist.main.10.79176c53yfCzKI&amp;algo_pvid=595eca82-0e86-47a6-9df1-3203eee67bde&amp;pdp_ext_f=%7B%22order%22%3A%22175%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A32676786935%7C_p_origin_prod%3A" xr:uid="{95FAB809-F896-4578-B2B0-BF3A464B12E5}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId12"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajustement taille trou face avant et base
</commit_message>
<xml_diff>
--- a/BOM_LignePassionIIm.xlsx
+++ b/BOM_LignePassionIIm.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/79fc430203973324/TravauxMetriques/IIm/Passion IIm/PupitreLigne/AlimLigne_PassionIIm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a43dc3239fed0de/PCB_Perso/PCB_IIm_Ligne/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="474" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F644F47C-1FCA-400C-B946-C6D87E7D66A8}"/>
+  <xr:revisionPtr revIDLastSave="475" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{486DE209-1E3B-49B9-A455-067AF7DA5B2A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -837,7 +837,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}" name="Tableau2" displayName="Tableau2" ref="A2:M36" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="3">
-  <autoFilter ref="A2:M36" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}"/>
+  <autoFilter ref="A2:M36" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}">
+    <filterColumn colId="10">
+      <filters>
+        <filter val="AliExpress"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:L36">
     <sortCondition ref="K2:K36"/>
   </sortState>
@@ -1180,20 +1186,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B7EC6F-57FE-4577-A1D4-89717E48955F}">
   <dimension ref="A1:M44"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="25.5703125" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" customWidth="1"/>
-    <col min="3" max="3" width="12.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" customWidth="1"/>
-    <col min="10" max="10" width="19.85546875" customWidth="1"/>
-    <col min="11" max="11" width="12.42578125" customWidth="1"/>
-    <col min="12" max="12" width="79.5703125" customWidth="1"/>
+    <col min="1" max="1" width="25.59765625" customWidth="1"/>
+    <col min="2" max="2" width="18.1328125" customWidth="1"/>
+    <col min="3" max="3" width="12.73046875" customWidth="1"/>
+    <col min="4" max="4" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.86328125" customWidth="1"/>
+    <col min="9" max="9" width="12.1328125" customWidth="1"/>
+    <col min="10" max="10" width="19.86328125" customWidth="1"/>
+    <col min="11" max="11" width="12.3984375" customWidth="1"/>
+    <col min="12" max="12" width="79.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="18" t="s">
         <v>26</v>
       </c>
@@ -1209,7 +1215,7 @@
       <c r="K1" s="18"/>
       <c r="L1" s="18"/>
     </row>
-    <row r="2" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
@@ -1250,7 +1256,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>57</v>
       </c>
@@ -1273,7 +1279,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -1295,7 +1301,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>105</v>
       </c>
@@ -1323,7 +1329,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>95</v>
       </c>
@@ -1351,7 +1357,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1376,7 +1382,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1401,7 +1407,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>63</v>
       </c>
@@ -1426,7 +1432,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>62</v>
       </c>
@@ -1451,7 +1457,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>71</v>
       </c>
@@ -1479,7 +1485,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>72</v>
       </c>
@@ -1501,7 +1507,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1523,7 +1529,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -1545,7 +1551,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>103</v>
       </c>
@@ -1567,7 +1573,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1600,7 +1606,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -1630,7 +1636,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>58</v>
       </c>
@@ -1652,7 +1658,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1677,7 +1683,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>555</v>
       </c>
@@ -1713,7 +1719,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1749,7 +1755,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1785,7 +1791,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -1821,7 +1827,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -1858,7 +1864,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>112</v>
       </c>
@@ -1892,7 +1898,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>84</v>
       </c>
@@ -1911,7 +1917,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -1935,7 +1941,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -1960,7 +1966,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1985,7 +1991,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -2010,7 +2016,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -2035,7 +2041,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -2060,7 +2066,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -2085,7 +2091,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2109,7 +2115,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>20</v>
       </c>
@@ -2129,7 +2135,7 @@
       </c>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2149,11 +2155,11 @@
       </c>
       <c r="J36" s="4"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A38" s="6" t="s">
         <v>29</v>
       </c>
@@ -2170,7 +2176,7 @@
       <c r="I38" s="2"/>
       <c r="J38" s="17"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A39" s="7" t="s">
         <v>28</v>
       </c>
@@ -2184,7 +2190,7 @@
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A40" s="7" t="s">
         <v>30</v>
       </c>
@@ -2196,7 +2202,7 @@
       <c r="E40" s="18"/>
       <c r="F40" s="23"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A41" s="10" t="s">
         <v>31</v>
       </c>
@@ -2208,15 +2214,15 @@
       <c r="E41" s="25"/>
       <c r="F41" s="26"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
     </row>

</xml_diff>

<commit_message>
Resistance de Shunt fix
</commit_message>
<xml_diff>
--- a/BOM_LignePassionIIm.xlsx
+++ b/BOM_LignePassionIIm.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7a43dc3239fed0de/PCB_Perso/PCB_IIm_Ligne/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="475" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{486DE209-1E3B-49B9-A455-067AF7DA5B2A}"/>
+  <xr:revisionPtr revIDLastSave="477" documentId="8_{D99A6803-265B-43E3-9609-960129D8CCE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7FA07D59-A12E-4907-8F0E-A2CAF75EACC1}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{C3AD9156-7CE6-4A1E-A3FD-D08ECF380023}"/>
   </bookViews>
@@ -837,13 +837,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}" name="Tableau2" displayName="Tableau2" ref="A2:M36" totalsRowShown="0" headerRowDxfId="4" headerRowBorderDxfId="3">
-  <autoFilter ref="A2:M36" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}">
-    <filterColumn colId="10">
-      <filters>
-        <filter val="AliExpress"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A2:M36" xr:uid="{69225E41-4DDD-470A-8E1A-242AA800D3ED}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:L36">
     <sortCondition ref="K2:K36"/>
   </sortState>
@@ -1573,7 +1567,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="16" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>8</v>
       </c>
@@ -1606,7 +1600,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -1636,7 +1630,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="18" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>58</v>
       </c>
@@ -1658,7 +1652,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1679,11 +1673,11 @@
       <c r="K19" t="s">
         <v>66</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L19" s="14" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" s="3">
         <v>555</v>
       </c>
@@ -1719,7 +1713,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>36</v>
       </c>
@@ -1755,7 +1749,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>40</v>
       </c>
@@ -1791,7 +1785,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>98</v>
       </c>
@@ -1827,7 +1821,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -1864,7 +1858,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>112</v>
       </c>
@@ -1898,7 +1892,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>84</v>
       </c>
@@ -1917,7 +1911,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>10</v>
       </c>
@@ -1941,7 +1935,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>20</v>
       </c>
@@ -1966,7 +1960,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1991,7 +1985,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>23</v>
       </c>
@@ -2016,7 +2010,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>23</v>
       </c>
@@ -2041,7 +2035,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>23</v>
       </c>
@@ -2066,7 +2060,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>23</v>
       </c>
@@ -2091,7 +2085,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>23</v>
       </c>
@@ -2115,7 +2109,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>20</v>
       </c>
@@ -2135,7 +2129,7 @@
       </c>
       <c r="J35" s="4"/>
     </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2235,11 +2229,12 @@
     <hyperlink ref="L16" r:id="rId1" xr:uid="{B3065FAB-E838-4A51-A82F-630335C42D81}"/>
     <hyperlink ref="L24" r:id="rId2" xr:uid="{2207D865-CE83-4458-802D-86175171E33D}"/>
     <hyperlink ref="L18" r:id="rId3" display="https://www.conrad.ch/de/p/tru-components-tc-13895648-rundsteckverbinder-stecker-buchsenkontakt-gesamtpolzahl-6-serie-rundsteckverbinder-gx16-3473912.html?insert=UP&amp;WT.srch=1&amp;ef_id=CjwKCAjw5s_QBhAdEiwADD_gBlB0NtPFlP1PxWWOBrmvbSo2JJn5T44wcE8r8-Hav4RDqu4GGAYJ1RoCRWEQAvD_BwE:G:s" xr:uid="{D4E7E61F-AE6E-48A3-9576-9A9FC4F56721}"/>
+    <hyperlink ref="L19" r:id="rId4" xr:uid="{FD97052D-7F57-49D4-BDD2-C0687DAB5CAD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId5"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>